<commit_message>
Build Henesys three-lane combat framework
</commit_message>
<xml_diff>
--- a/ExcelTable/Combat.xlsx
+++ b/ExcelTable/Combat.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatConfig" sheetId="1" r:id="R6dbab857c6d0425a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuntingGroundTiers" sheetId="2" r:id="R282fff0cd8ba4c85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="3" r:id="R9b989a8efc2d4584"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterDefinitions" sheetId="4" r:id="R11e1f275586a4e08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpawnGroups" sheetId="5" r:id="Rfffa170c7b614104"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatConfig" sheetId="1" r:id="Rd69644962b5e4b59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuntingGroundTiers" sheetId="2" r:id="R6092f6b4ea0c463a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="3" r:id="R337c2822b9514937"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterDefinitions" sheetId="4" r:id="R3ab787fc229c4482"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpawnGroups" sheetId="5" r:id="Raf0ce2c49ab04c32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLanes" sheetId="6" r:id="Raf813a77ff0b48e5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,12 +56,62 @@
       <x:name val="Malgun Gothic"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF172033"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF334155"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2E8F0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF172033"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF334155"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2E8F0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -108,7 +159,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="19">
+  <x:cellXfs count="43">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
@@ -160,6 +211,46 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -385,6 +476,15 @@
     <x:col min="4" max="4" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="23.75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.5" customHeight="1">
@@ -406,6 +506,33 @@
       <x:c r="F1" s="7" t="str">
         <x:v>RuntimeKind</x:v>
       </x:c>
+      <x:c r="G1" s="20" t="str">
+        <x:v>HenesysMapKey</x:v>
+      </x:c>
+      <x:c r="H1" s="20" t="str">
+        <x:v>LaneMatchTolerance</x:v>
+      </x:c>
+      <x:c r="I1" s="20" t="str">
+        <x:v>MinimumLaneSpacing</x:v>
+      </x:c>
+      <x:c r="J1" s="20" t="str">
+        <x:v>PlayerSpawnNormalizedX</x:v>
+      </x:c>
+      <x:c r="K1" s="20" t="str">
+        <x:v>MonsterSpawnNormalizedX</x:v>
+      </x:c>
+      <x:c r="L1" s="20" t="str">
+        <x:v>CombatBoundsInset</x:v>
+      </x:c>
+      <x:c r="M1" s="20" t="str">
+        <x:v>PlayerSpawnYOffset</x:v>
+      </x:c>
+      <x:c r="N1" s="33" t="str">
+        <x:v>CombatAreaMinimumWorldX</x:v>
+      </x:c>
+      <x:c r="O1" s="33" t="str">
+        <x:v>CombatAreaMaximumWorldX</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -425,6 +552,33 @@
       </x:c>
       <x:c r="F2" s="9" t="str">
         <x:v>all</x:v>
+      </x:c>
+      <x:c r="G2" s="22" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="H2" s="22" t="str">
+        <x:v>design</x:v>
+      </x:c>
+      <x:c r="I2" s="22" t="str">
+        <x:v>design</x:v>
+      </x:c>
+      <x:c r="J2" s="22" t="str">
+        <x:v>design</x:v>
+      </x:c>
+      <x:c r="K2" s="22" t="str">
+        <x:v>design</x:v>
+      </x:c>
+      <x:c r="L2" s="22" t="str">
+        <x:v>design</x:v>
+      </x:c>
+      <x:c r="M2" s="22" t="str">
+        <x:v>design</x:v>
+      </x:c>
+      <x:c r="N2" s="35" t="str">
+        <x:v>design</x:v>
+      </x:c>
+      <x:c r="O2" s="35" t="str">
+        <x:v>design</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
@@ -446,6 +600,33 @@
       <x:c r="F3" s="12" t="str">
         <x:v>전투 하네스가 활성화될 런타임 구분 값입니다.</x:v>
       </x:c>
+      <x:c r="G3" s="25" t="str">
+        <x:v>헤네시스 3층 전투 구역을 배치할 맵 키입니다.</x:v>
+      </x:c>
+      <x:c r="H3" s="25" t="str">
+        <x:v>발판 Y와 CombatLanes.WorldYOffset의 허용 오차입니다.</x:v>
+      </x:c>
+      <x:c r="I3" s="25" t="str">
+        <x:v>인접한 전투 층 사이의 최소 세로 간격입니다.</x:v>
+      </x:c>
+      <x:c r="J3" s="25" t="str">
+        <x:v>공통 발판 폭침에서 플레이어가 스폰할 0~1 가로 비율입니다.</x:v>
+      </x:c>
+      <x:c r="K3" s="25" t="str">
+        <x:v>공통 발판 폭침에서 몬스터가 스폰할 0~1 가로 비율입니다.</x:v>
+      </x:c>
+      <x:c r="L3" s="25" t="str">
+        <x:v>발판 양쪽 끝에서 전투 범위를 안쪽으로 줄이는 거리입니다.</x:v>
+      </x:c>
+      <x:c r="M3" s="25" t="str">
+        <x:v>중앙층 발판 위로 플레이어를 올릴 Y 오프셋입니다.</x:v>
+      </x:c>
+      <x:c r="N3" s="38" t="str">
+        <x:v>화면 오른쪽 전투 구역의 최소 세계 X 좌표입니다.</x:v>
+      </x:c>
+      <x:c r="O3" s="38" t="str">
+        <x:v>화면 오른쪽 전투 구역의 최대 세계 X 좌표입니다.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -465,6 +646,33 @@
       </x:c>
       <x:c r="F4" s="14" t="str">
         <x:v>string</x:v>
+      </x:c>
+      <x:c r="G4" s="27" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="H4" s="27" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="I4" s="27" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="J4" s="27" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="K4" s="27" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="L4" s="27" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="M4" s="27" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="N4" s="40" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="O4" s="40" t="str">
+        <x:v>float</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
@@ -484,7 +692,34 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F5" s="17" t="str">
-        <x:v>TEST_SANDBOX</x:v>
+        <x:v>HENESYS_TILE_LANES</x:v>
+      </x:c>
+      <x:c r="G5" s="29" t="str">
+        <x:v>map01</x:v>
+      </x:c>
+      <x:c r="H5" s="29" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
+      <x:c r="I5" s="29" t="n">
+        <x:v>1.8</x:v>
+      </x:c>
+      <x:c r="J5" s="29" t="n">
+        <x:v>0.32</x:v>
+      </x:c>
+      <x:c r="K5" s="29" t="n">
+        <x:v>0.68</x:v>
+      </x:c>
+      <x:c r="L5" s="29" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="M5" s="29" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="N5" s="42" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O5" s="42" t="n">
+        <x:v>8</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -641,6 +876,8 @@
     <x:col min="10" max="10" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="32.5" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="18.1299991607666" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.5" customHeight="1">
@@ -680,6 +917,12 @@
       <x:c r="L1" s="7" t="str">
         <x:v>Notes</x:v>
       </x:c>
+      <x:c r="M1" s="20" t="str">
+        <x:v>BasicAttackLaneKey</x:v>
+      </x:c>
+      <x:c r="N1" s="20" t="str">
+        <x:v>AttackHitboxHeight</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -717,6 +960,12 @@
       </x:c>
       <x:c r="L2" s="9" t="str">
         <x:v>design</x:v>
+      </x:c>
+      <x:c r="M2" s="22" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="N2" s="22" t="str">
+        <x:v>server</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
@@ -756,6 +1005,12 @@
       <x:c r="L3" s="12" t="str">
         <x:v>기획 참고 메모입니다.</x:v>
       </x:c>
+      <x:c r="M3" s="25" t="str">
+        <x:v>기본 공격과 초반 스킬이 타격할 전투 층 키입니다.</x:v>
+      </x:c>
+      <x:c r="N3" s="25" t="str">
+        <x:v>기본 공격 히트박스의 세로 크기입니다.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -794,6 +1049,12 @@
       <x:c r="L4" s="14" t="str">
         <x:v>string</x:v>
       </x:c>
+      <x:c r="M4" s="27" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="N4" s="27" t="str">
+        <x:v>float</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
       <x:c r="A5" s="17" t="n">
@@ -831,6 +1092,12 @@
       </x:c>
       <x:c r="L5" s="17" t="str">
         <x:v>Initial auto-battle profile</x:v>
+      </x:c>
+      <x:c r="M5" s="29" t="str">
+        <x:v>CENTER</x:v>
+      </x:c>
+      <x:c r="N5" s="29" t="n">
+        <x:v>1.2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -861,6 +1128,7 @@
     <x:col min="17" max="17" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="32.5" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="18.1299991607666" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.5" customHeight="1">
@@ -921,6 +1189,9 @@
       <x:c r="S1" s="7" t="str">
         <x:v>Notes</x:v>
       </x:c>
+      <x:c r="T1" s="20" t="str">
+        <x:v>AttackHitboxHeight</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -979,6 +1250,9 @@
       </x:c>
       <x:c r="S2" s="9" t="str">
         <x:v>design</x:v>
+      </x:c>
+      <x:c r="T2" s="22" t="str">
+        <x:v>server</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
@@ -1039,6 +1313,9 @@
       <x:c r="S3" s="12" t="str">
         <x:v>기획 참고 메모입니다.</x:v>
       </x:c>
+      <x:c r="T3" s="25" t="str">
+        <x:v>몬스터 공격 히트박스의 세로 크기입니다.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -1098,6 +1375,9 @@
       <x:c r="S4" s="14" t="str">
         <x:v>string</x:v>
       </x:c>
+      <x:c r="T4" s="27" t="str">
+        <x:v>float</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
       <x:c r="A5" s="17" t="n">
@@ -1156,6 +1436,9 @@
       </x:c>
       <x:c r="S5" s="17" t="str">
         <x:v>Classic Tier 1 Slime</x:v>
+      </x:c>
+      <x:c r="T5" s="29" t="n">
+        <x:v>1.2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1177,6 +1460,7 @@
     <x:col min="8" max="8" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="32.5" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23.75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.5" customHeight="1">
@@ -1210,6 +1494,9 @@
       <x:c r="J1" s="7" t="str">
         <x:v>Notes</x:v>
       </x:c>
+      <x:c r="K1" s="20" t="str">
+        <x:v>LaneKey</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -1241,6 +1528,9 @@
       </x:c>
       <x:c r="J2" s="9" t="str">
         <x:v>design</x:v>
+      </x:c>
+      <x:c r="K2" s="22" t="str">
+        <x:v>server</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
@@ -1274,6 +1564,9 @@
       <x:c r="J3" s="12" t="str">
         <x:v>기획 참고 메모입니다.</x:v>
       </x:c>
+      <x:c r="K3" s="25" t="str">
+        <x:v>해당 스폰 그룹이 속한 전투 층 키입니다.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -1306,6 +1599,9 @@
       <x:c r="J4" s="14" t="str">
         <x:v>string</x:v>
       </x:c>
+      <x:c r="K4" s="27" t="str">
+        <x:v>string</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
       <x:c r="A5" s="17" t="n">
@@ -1321,13 +1617,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E5" s="17" t="str">
-        <x:v>CombatHarness/MonsterSpawn/Tier1</x:v>
+        <x:v>CombatHarness/Lanes/CENTER/Spawn</x:v>
       </x:c>
       <x:c r="F5" s="17" t="str">
-        <x:v>CombatHarness/CombatBoundsLeft</x:v>
+        <x:v>CombatHarness/Lanes/CENTER/BoundsLeft</x:v>
       </x:c>
       <x:c r="G5" s="17" t="str">
-        <x:v>CombatHarness/CombatBoundsRight</x:v>
+        <x:v>CombatHarness/Lanes/CENTER/BoundsRight</x:v>
       </x:c>
       <x:c r="H5" s="17" t="n">
         <x:v>0.4</x:v>
@@ -1337,6 +1633,342 @@
       </x:c>
       <x:c r="J5" s="17" t="str">
         <x:v>Single Slime foundation group</x:v>
+      </x:c>
+      <x:c r="K5" s="29" t="str">
+        <x:v>CENTER</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="32.5" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="16.5" customHeight="1">
+      <x:c r="A1" s="20" t="str">
+        <x:v>CombatLanesIndex</x:v>
+      </x:c>
+      <x:c r="B1" s="20" t="str">
+        <x:v>HuntingGroundTierIndex</x:v>
+      </x:c>
+      <x:c r="C1" s="20" t="str">
+        <x:v>MapKey</x:v>
+      </x:c>
+      <x:c r="D1" s="20" t="str">
+        <x:v>LaneKey</x:v>
+      </x:c>
+      <x:c r="E1" s="20" t="str">
+        <x:v>LaneOrder</x:v>
+      </x:c>
+      <x:c r="F1" s="20" t="str">
+        <x:v>WorldYOffset</x:v>
+      </x:c>
+      <x:c r="G1" s="20" t="str">
+        <x:v>MinimumHorizontalSpan</x:v>
+      </x:c>
+      <x:c r="H1" s="20" t="str">
+        <x:v>BasicAttackTargetable</x:v>
+      </x:c>
+      <x:c r="I1" s="20" t="str">
+        <x:v>InitialSpawnEnabled</x:v>
+      </x:c>
+      <x:c r="J1" s="20" t="str">
+        <x:v>SpawnAnchorKey</x:v>
+      </x:c>
+      <x:c r="K1" s="20" t="str">
+        <x:v>BoundsLeftAnchorKey</x:v>
+      </x:c>
+      <x:c r="L1" s="20" t="str">
+        <x:v>BoundsRightAnchorKey</x:v>
+      </x:c>
+      <x:c r="M1" s="20" t="str">
+        <x:v>Enabled</x:v>
+      </x:c>
+      <x:c r="N1" s="20" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="16.5" customHeight="1">
+      <x:c r="A2" s="22" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="B2" s="22" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="C2" s="22" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="D2" s="22" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="E2" s="22" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="F2" s="22" t="str">
+        <x:v>design</x:v>
+      </x:c>
+      <x:c r="G2" s="22" t="str">
+        <x:v>design</x:v>
+      </x:c>
+      <x:c r="H2" s="22" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="I2" s="22" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="J2" s="22" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="K2" s="22" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="L2" s="22" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="M2" s="22" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="N2" s="22" t="str">
+        <x:v>design</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1">
+      <x:c r="A3" s="25" t="str">
+        <x:v>전투 층 행을 식별하는 인덱스입니다.</x:v>
+      </x:c>
+      <x:c r="B3" s="25" t="str">
+        <x:v>HuntingGroundTiers를 참조하는 인덱스입니다.</x:v>
+      </x:c>
+      <x:c r="C3" s="25" t="str">
+        <x:v>이 전투 층이 속한 맵 키입니다.</x:v>
+      </x:c>
+      <x:c r="D3" s="25" t="str">
+        <x:v>UPPER, CENTER, LOWER 중 하나인 고정 층 키입니다.</x:v>
+      </x:c>
+      <x:c r="E3" s="25" t="str">
+        <x:v>위에서 아래로 정렬하는 1기반 순서입니다.</x:v>
+      </x:c>
+      <x:c r="F3" s="25" t="str">
+        <x:v>CENTER를 0으로 본 예상 세계 Y 오프셋입니다.</x:v>
+      </x:c>
+      <x:c r="G3" s="25" t="str">
+        <x:v>해당 층 발판이 가져야 할 최소 가로 길이입니다.</x:v>
+      </x:c>
+      <x:c r="H3" s="25" t="str">
+        <x:v>기본 공격과 초반 스킬이 해당 층을 타격할 수 있는지 여부입니다.</x:v>
+      </x:c>
+      <x:c r="I3" s="25" t="str">
+        <x:v>초기 헤네시스 진입 시 이 층에 몬스터를 배치할지 여부입니다.</x:v>
+      </x:c>
+      <x:c r="J3" s="25" t="str">
+        <x:v>해당 층 몬스터 스폰 앵커 경로입니다.</x:v>
+      </x:c>
+      <x:c r="K3" s="25" t="str">
+        <x:v>해당 층 전투 범위 왼쪽 앵커 경로입니다.</x:v>
+      </x:c>
+      <x:c r="L3" s="25" t="str">
+        <x:v>해당 층 전투 범위 오른쪽 앵커 경로입니다.</x:v>
+      </x:c>
+      <x:c r="M3" s="25" t="str">
+        <x:v>해당 전투 층을 사용할지 여부입니다.</x:v>
+      </x:c>
+      <x:c r="N3" s="25" t="str">
+        <x:v>기획 참고 메모입니다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="16.5" customHeight="1">
+      <x:c r="A4" s="27" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="B4" s="27" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="C4" s="27" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D4" s="27" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="E4" s="27" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="F4" s="27" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="G4" s="27" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="H4" s="27" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+      <x:c r="I4" s="27" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+      <x:c r="J4" s="27" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="K4" s="27" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="L4" s="27" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="M4" s="27" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+      <x:c r="N4" s="27" t="str">
+        <x:v>string</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="16.5" customHeight="1">
+      <x:c r="A5" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C5" s="29" t="str">
+        <x:v>map01</x:v>
+      </x:c>
+      <x:c r="D5" s="29" t="str">
+        <x:v>UPPER</x:v>
+      </x:c>
+      <x:c r="E5" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F5" s="29" t="n">
+        <x:v>2.1</x:v>
+      </x:c>
+      <x:c r="G5" s="29" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H5" s="31" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I5" s="31" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J5" s="29" t="str">
+        <x:v>CombatHarness/Lanes/UPPER/Spawn</x:v>
+      </x:c>
+      <x:c r="K5" s="29" t="str">
+        <x:v>CombatHarness/Lanes/UPPER/BoundsLeft</x:v>
+      </x:c>
+      <x:c r="L5" s="29" t="str">
+        <x:v>CombatHarness/Lanes/UPPER/BoundsRight</x:v>
+      </x:c>
+      <x:c r="M5" s="31" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N5" s="29" t="str">
+        <x:v>Future upper-lane area skill target</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="16.5" customHeight="1">
+      <x:c r="A6" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" s="29" t="str">
+        <x:v>map01</x:v>
+      </x:c>
+      <x:c r="D6" s="29" t="str">
+        <x:v>CENTER</x:v>
+      </x:c>
+      <x:c r="E6" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F6" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G6" s="29" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H6" s="31" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I6" s="31" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J6" s="29" t="str">
+        <x:v>CombatHarness/Lanes/CENTER/Spawn</x:v>
+      </x:c>
+      <x:c r="K6" s="29" t="str">
+        <x:v>CombatHarness/Lanes/CENTER/BoundsLeft</x:v>
+      </x:c>
+      <x:c r="L6" s="29" t="str">
+        <x:v>CombatHarness/Lanes/CENTER/BoundsRight</x:v>
+      </x:c>
+      <x:c r="M6" s="31" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N6" s="29" t="str">
+        <x:v>Initial basic attack hunting lane</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="16.5" customHeight="1">
+      <x:c r="A7" s="29" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="29" t="str">
+        <x:v>map01</x:v>
+      </x:c>
+      <x:c r="D7" s="29" t="str">
+        <x:v>LOWER</x:v>
+      </x:c>
+      <x:c r="E7" s="29" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F7" s="29" t="n">
+        <x:v>-2.1</x:v>
+      </x:c>
+      <x:c r="G7" s="29" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H7" s="31" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I7" s="31" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J7" s="29" t="str">
+        <x:v>CombatHarness/Lanes/LOWER/Spawn</x:v>
+      </x:c>
+      <x:c r="K7" s="29" t="str">
+        <x:v>CombatHarness/Lanes/LOWER/BoundsLeft</x:v>
+      </x:c>
+      <x:c r="L7" s="29" t="str">
+        <x:v>CombatHarness/Lanes/LOWER/BoundsRight</x:v>
+      </x:c>
+      <x:c r="M7" s="31" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N7" s="29" t="str">
+        <x:v>Future lower-lane area skill target</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Place Henesys three-lane combat harness
</commit_message>
<xml_diff>
--- a/ExcelTable/Combat.xlsx
+++ b/ExcelTable/Combat.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatConfig" sheetId="1" r:id="Rd69644962b5e4b59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuntingGroundTiers" sheetId="2" r:id="R6092f6b4ea0c463a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="3" r:id="R337c2822b9514937"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterDefinitions" sheetId="4" r:id="R3ab787fc229c4482"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpawnGroups" sheetId="5" r:id="Raf0ce2c49ab04c32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLanes" sheetId="6" r:id="Raf813a77ff0b48e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatConfig" sheetId="1" r:id="Rb1ac1552019f4f4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuntingGroundTiers" sheetId="2" r:id="R3066aaa331c94c75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="3" r:id="R6dcb9f8dc1f443b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterDefinitions" sheetId="4" r:id="R470927d8af184716"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpawnGroups" sheetId="5" r:id="R81d4c1eb5ab64c8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLanes" sheetId="6" r:id="Rf83562a1f6ef445e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1859,7 +1859,7 @@
         <x:v>2.1</x:v>
       </x:c>
       <x:c r="G5" s="29" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H5" s="31" t="b">
         <x:v>0</x:v>
@@ -1903,7 +1903,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G6" s="29" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H6" s="31" t="b">
         <x:v>1</x:v>
@@ -1947,7 +1947,7 @@
         <x:v>-2.1</x:v>
       </x:c>
       <x:c r="G7" s="29" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H7" s="31" t="b">
         <x:v>0</x:v>

</xml_diff>

<commit_message>
Fix combat input and camera composition
</commit_message>
<xml_diff>
--- a/ExcelTable/Combat.xlsx
+++ b/ExcelTable/Combat.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatConfig" sheetId="1" r:id="Rb1ac1552019f4f4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuntingGroundTiers" sheetId="2" r:id="R3066aaa331c94c75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="3" r:id="R6dcb9f8dc1f443b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterDefinitions" sheetId="4" r:id="R470927d8af184716"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpawnGroups" sheetId="5" r:id="R81d4c1eb5ab64c8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLanes" sheetId="6" r:id="Rf83562a1f6ef445e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatConfig" sheetId="1" r:id="Rad97b8f0bc5948aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuntingGroundTiers" sheetId="2" r:id="R57b4c96b8b5a4ef2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="3" r:id="R03b2e695a704449e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterDefinitions" sheetId="4" r:id="R4d592528fdc147d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpawnGroups" sheetId="5" r:id="R671b50bc59e44c7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLanes" sheetId="6" r:id="Re2be16a24dd247f4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -56,12 +56,37 @@
       <x:name val="Malgun Gothic"/>
     </x:font>
   </x:fonts>
-  <x:fills count="17">
+  <x:fills count="22">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF172033"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF334155"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2E8F0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -159,7 +184,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="43">
+  <x:cellXfs count="56">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
@@ -251,6 +276,33 @@
     <x:xf numFmtId="0" fontId="5" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -485,6 +537,9 @@
     <x:col min="13" max="13" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="23.75" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="23.75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.5" customHeight="1">
@@ -533,6 +588,15 @@
       <x:c r="O1" s="33" t="str">
         <x:v>CombatAreaMaximumWorldX</x:v>
       </x:c>
+      <x:c r="P1" s="44" t="str">
+        <x:v>CombatCameraScreenOffsetX</x:v>
+      </x:c>
+      <x:c r="Q1" s="44" t="str">
+        <x:v>CombatCameraScreenOffsetY</x:v>
+      </x:c>
+      <x:c r="R1" s="44" t="str">
+        <x:v>CombatCameraConfineArea</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -578,6 +642,15 @@
         <x:v>design</x:v>
       </x:c>
       <x:c r="O2" s="35" t="str">
+        <x:v>design</x:v>
+      </x:c>
+      <x:c r="P2" s="46" t="str">
+        <x:v>design</x:v>
+      </x:c>
+      <x:c r="Q2" s="46" t="str">
+        <x:v>design</x:v>
+      </x:c>
+      <x:c r="R2" s="46" t="str">
         <x:v>design</x:v>
       </x:c>
     </x:row>
@@ -627,6 +700,15 @@
       <x:c r="O3" s="38" t="str">
         <x:v>화면 오른쪽 전투 구역의 최대 세계 X 좌표입니다.</x:v>
       </x:c>
+      <x:c r="P3" s="49" t="str">
+        <x:v>전투 중 플레이어가 화면 가로에서 표시될 0~1 비율입니다.</x:v>
+      </x:c>
+      <x:c r="Q3" s="49" t="str">
+        <x:v>전투 중 플레이어가 화면 세로에서 표시될 0~1 비율입니다.</x:v>
+      </x:c>
+      <x:c r="R3" s="49" t="str">
+        <x:v>전투 중 카메라를 발판 영역에 자동 구속할지 여부입니다.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -673,6 +755,15 @@
       </x:c>
       <x:c r="O4" s="40" t="str">
         <x:v>float</x:v>
+      </x:c>
+      <x:c r="P4" s="51" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="Q4" s="51" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="R4" s="51" t="str">
+        <x:v>bool</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
@@ -720,6 +811,15 @@
       </x:c>
       <x:c r="O5" s="42" t="n">
         <x:v>8</x:v>
+      </x:c>
+      <x:c r="P5" s="53" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="Q5" s="53" t="n">
+        <x:v>0.655</x:v>
+      </x:c>
+      <x:c r="R5" s="55" t="b">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Use fixed camera for Henesys combat
</commit_message>
<xml_diff>
--- a/ExcelTable/Combat.xlsx
+++ b/ExcelTable/Combat.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatConfig" sheetId="1" r:id="Rad97b8f0bc5948aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuntingGroundTiers" sheetId="2" r:id="R57b4c96b8b5a4ef2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="3" r:id="R03b2e695a704449e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterDefinitions" sheetId="4" r:id="R4d592528fdc147d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpawnGroups" sheetId="5" r:id="R671b50bc59e44c7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLanes" sheetId="6" r:id="Re2be16a24dd247f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatConfig" sheetId="1" r:id="R54b3c91f24294dd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuntingGroundTiers" sheetId="2" r:id="R978787b82a024461"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="3" r:id="R5a80b5b29900436b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterDefinitions" sheetId="4" r:id="R517050060b504bd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpawnGroups" sheetId="5" r:id="Rcf2faea0cdf34c6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLanes" sheetId="6" r:id="Rdc7a5315e7a544c9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -56,12 +56,37 @@
       <x:name val="Malgun Gothic"/>
     </x:font>
   </x:fonts>
-  <x:fills count="22">
+  <x:fills count="27">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF172033"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF334155"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2E8F0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -184,7 +209,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="56">
+  <x:cellXfs count="67">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
@@ -303,6 +328,19 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="23" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="24" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="24" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="25" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="25" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="26" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="26" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -540,6 +578,7 @@
     <x:col min="16" max="16" width="23.75" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="23.75" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="23.75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.5" customHeight="1">
@@ -597,6 +636,9 @@
       <x:c r="R1" s="44" t="str">
         <x:v>CombatCameraConfineArea</x:v>
       </x:c>
+      <x:c r="S1" s="57" t="str">
+        <x:v>CombatCameraAnchorKey</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -652,6 +694,9 @@
       </x:c>
       <x:c r="R2" s="46" t="str">
         <x:v>design</x:v>
+      </x:c>
+      <x:c r="S2" s="59" t="str">
+        <x:v>all</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
@@ -701,14 +746,17 @@
         <x:v>화면 오른쪽 전투 구역의 최대 세계 X 좌표입니다.</x:v>
       </x:c>
       <x:c r="P3" s="49" t="str">
-        <x:v>전투 중 플레이어가 화면 가로에서 표시될 0~1 비율입니다.</x:v>
+        <x:v>전투 중 고정 카메라 앵커가 화면 가로에서 표시될 0~1 비율입니다.</x:v>
       </x:c>
       <x:c r="Q3" s="49" t="str">
-        <x:v>전투 중 플레이어가 화면 세로에서 표시될 0~1 비율입니다.</x:v>
+        <x:v>전투 중 고정 카메라 앵커가 화면 세로에서 표시될 0~1 비율입니다.</x:v>
       </x:c>
       <x:c r="R3" s="49" t="str">
         <x:v>전투 중 카메라를 발판 영역에 자동 구속할지 여부입니다.</x:v>
       </x:c>
+      <x:c r="S3" s="62" t="str">
+        <x:v>발판 공통 중앙에 배치할 고정 전투 카메라 앵커 경로입니다.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -764,6 +812,9 @@
       </x:c>
       <x:c r="R4" s="51" t="str">
         <x:v>bool</x:v>
+      </x:c>
+      <x:c r="S4" s="64" t="str">
+        <x:v>string</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
@@ -820,6 +871,9 @@
       </x:c>
       <x:c r="R5" s="55" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="S5" s="66" t="str">
+        <x:v>CombatHarness/CameraAnchor</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Implement runtime Henesys auto battle
</commit_message>
<xml_diff>
--- a/ExcelTable/Combat.xlsx
+++ b/ExcelTable/Combat.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatConfig" sheetId="1" r:id="R54b3c91f24294dd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuntingGroundTiers" sheetId="2" r:id="R978787b82a024461"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="3" r:id="R5a80b5b29900436b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterDefinitions" sheetId="4" r:id="R517050060b504bd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpawnGroups" sheetId="5" r:id="Rcf2faea0cdf34c6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLanes" sheetId="6" r:id="Rdc7a5315e7a544c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatConfig" sheetId="1" r:id="R0e1654f725264d10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuntingGroundTiers" sheetId="2" r:id="R27932cf5a07240db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="3" r:id="Ra234e03ea7634607"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterDefinitions" sheetId="4" r:id="R6f2e9165c9fa4e13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpawnGroups" sheetId="5" r:id="R9cd433e1ad85499d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLanes" sheetId="6" r:id="Rbe446bdc15774c23"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2013,7 +2013,7 @@
         <x:v>2.1</x:v>
       </x:c>
       <x:c r="G5" s="29" t="n">
-        <x:v>5</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="H5" s="31" t="b">
         <x:v>0</x:v>
@@ -2057,7 +2057,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G6" s="29" t="n">
-        <x:v>5</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="H6" s="31" t="b">
         <x:v>1</x:v>
@@ -2101,7 +2101,7 @@
         <x:v>-2.1</x:v>
       </x:c>
       <x:c r="G7" s="29" t="n">
-        <x:v>5</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="H7" s="31" t="b">
         <x:v>0</x:v>

</xml_diff>

<commit_message>
Fix map-wide auto battle targeting and contact damage
</commit_message>
<xml_diff>
--- a/ExcelTable/Combat.xlsx
+++ b/ExcelTable/Combat.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatConfig" sheetId="1" r:id="R0e1654f725264d10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuntingGroundTiers" sheetId="2" r:id="R27932cf5a07240db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="3" r:id="Ra234e03ea7634607"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterDefinitions" sheetId="4" r:id="R6f2e9165c9fa4e13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpawnGroups" sheetId="5" r:id="R9cd433e1ad85499d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLanes" sheetId="6" r:id="Rbe446bdc15774c23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatConfig" sheetId="1" r:id="Rfcc5ab25b8b24da9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuntingGroundTiers" sheetId="2" r:id="Ra9be36f89ce84f81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="3" r:id="Rff49519869bd44a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterDefinitions" sheetId="4" r:id="R74c31bae12234484"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpawnGroups" sheetId="5" r:id="R10515a0c3b954055"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLanes" sheetId="6" r:id="R35da22f3aeaa43df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLadders" sheetId="7" r:id="R54941e00c2e14a8c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -56,12 +57,37 @@
       <x:name val="Malgun Gothic"/>
     </x:font>
   </x:fonts>
-  <x:fills count="27">
+  <x:fills count="32">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF172033"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF334155"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2E8F0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -209,7 +235,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="67">
+  <x:cellXfs count="80">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
@@ -341,6 +367,33 @@
     <x:xf numFmtId="0" fontId="5" fillId="25" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="26" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="26" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="27" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="27" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="28" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="28" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="29" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="29" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="29" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="30" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="30" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="31" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="31" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="31" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="31" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1032,6 +1085,8 @@
     <x:col min="12" max="12" width="32.5" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="23.75" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="23.75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.5" customHeight="1">
@@ -1077,6 +1132,12 @@
       <x:c r="N1" s="20" t="str">
         <x:v>AttackHitboxHeight</x:v>
       </x:c>
+      <x:c r="O1" s="68" t="str">
+        <x:v>LadderApproachTolerance</x:v>
+      </x:c>
+      <x:c r="P1" s="68" t="str">
+        <x:v>LadderExitTolerance</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -1119,6 +1180,12 @@
         <x:v>server</x:v>
       </x:c>
       <x:c r="N2" s="22" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="O2" s="70" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="P2" s="70" t="str">
         <x:v>server</x:v>
       </x:c>
     </x:row>
@@ -1165,6 +1232,12 @@
       <x:c r="N3" s="25" t="str">
         <x:v>기본 공격 히트박스의 세로 크기입니다.</x:v>
       </x:c>
+      <x:c r="O3" s="73" t="str">
+        <x:v>사다리 중앙에 도착했다고 보는 가로 허용 거리입니다.</x:v>
+      </x:c>
+      <x:c r="P3" s="73" t="str">
+        <x:v>목표 층에 도착했다고 보는 세로 허용 거리입니다.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -1209,6 +1282,12 @@
       <x:c r="N4" s="27" t="str">
         <x:v>float</x:v>
       </x:c>
+      <x:c r="O4" s="75" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="P4" s="75" t="str">
+        <x:v>float</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
       <x:c r="A5" s="17" t="n">
@@ -1239,19 +1318,25 @@
         <x:v>1500</x:v>
       </x:c>
       <x:c r="J5" s="17" t="n">
-        <x:v>8</x:v>
+        <x:v>9999</x:v>
       </x:c>
       <x:c r="K5" s="18" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L5" s="17" t="str">
-        <x:v>Initial auto-battle profile</x:v>
+        <x:v>Map-wide ladder auto-battle profile</x:v>
       </x:c>
       <x:c r="M5" s="29" t="str">
         <x:v>CENTER</x:v>
       </x:c>
       <x:c r="N5" s="29" t="n">
         <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="O5" s="77" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
+      <x:c r="P5" s="77" t="n">
+        <x:v>0.25</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1283,6 +1368,14 @@
     <x:col min="18" max="18" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="32.5" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="35" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="23.75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.5" customHeight="1">
@@ -1346,6 +1439,30 @@
       <x:c r="T1" s="20" t="str">
         <x:v>AttackHitboxHeight</x:v>
       </x:c>
+      <x:c r="U1" s="68" t="str">
+        <x:v>AttackAnimationRuid</x:v>
+      </x:c>
+      <x:c r="V1" s="68" t="str">
+        <x:v>AttackMode</x:v>
+      </x:c>
+      <x:c r="W1" s="68" t="str">
+        <x:v>Aggressive</x:v>
+      </x:c>
+      <x:c r="X1" s="68" t="str">
+        <x:v>IdleMinSeconds</x:v>
+      </x:c>
+      <x:c r="Y1" s="68" t="str">
+        <x:v>IdleMaxSeconds</x:v>
+      </x:c>
+      <x:c r="Z1" s="68" t="str">
+        <x:v>WanderMinSeconds</x:v>
+      </x:c>
+      <x:c r="AA1" s="68" t="str">
+        <x:v>WanderMaxSeconds</x:v>
+      </x:c>
+      <x:c r="AB1" s="68" t="str">
+        <x:v>ContactMoveThroughSeconds</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -1406,6 +1523,30 @@
         <x:v>design</x:v>
       </x:c>
       <x:c r="T2" s="22" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="U2" s="70" t="str">
+        <x:v>client</x:v>
+      </x:c>
+      <x:c r="V2" s="70" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="W2" s="70" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="X2" s="70" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="Y2" s="70" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="Z2" s="70" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="AA2" s="70" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="AB2" s="70" t="str">
         <x:v>server</x:v>
       </x:c>
     </x:row>
@@ -1470,6 +1611,30 @@
       <x:c r="T3" s="25" t="str">
         <x:v>몬스터 공격 히트박스의 세로 크기입니다.</x:v>
       </x:c>
+      <x:c r="U3" s="73" t="str">
+        <x:v>능동 공격 애니메이션 RUID이며 접촉형은 비워둡니다.</x:v>
+      </x:c>
+      <x:c r="V3" s="73" t="str">
+        <x:v>CONTACT 또는 ACTIVE 공격 방식입니다.</x:v>
+      </x:c>
+      <x:c r="W3" s="73" t="str">
+        <x:v>플레이어를 먼저 발견하면 추격하는 선공 여부입니다.</x:v>
+      </x:c>
+      <x:c r="X3" s="73" t="str">
+        <x:v>자율 대기 최소 시간입니다.</x:v>
+      </x:c>
+      <x:c r="Y3" s="73" t="str">
+        <x:v>자율 대기 최대 시간입니다.</x:v>
+      </x:c>
+      <x:c r="Z3" s="73" t="str">
+        <x:v>자율 이동 최소 시간입니다.</x:v>
+      </x:c>
+      <x:c r="AA3" s="73" t="str">
+        <x:v>자율 이동 최대 시간입니다.</x:v>
+      </x:c>
+      <x:c r="AB3" s="73" t="str">
+        <x:v>접촉 피해 후 기존 방향으로 계속 이동하는 시간입니다.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -1532,6 +1697,30 @@
       <x:c r="T4" s="27" t="str">
         <x:v>float</x:v>
       </x:c>
+      <x:c r="U4" s="75" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="V4" s="75" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="W4" s="75" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+      <x:c r="X4" s="75" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="Y4" s="75" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="Z4" s="75" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="AA4" s="75" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="AB4" s="75" t="str">
+        <x:v>float</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
       <x:c r="A5" s="17" t="n">
@@ -1577,22 +1766,130 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="O5" s="17" t="n">
-        <x:v>1.1</x:v>
+        <x:v>0.65</x:v>
       </x:c>
       <x:c r="P5" s="17" t="str">
         <x:v>DROP_SLIME_TIER1</x:v>
       </x:c>
       <x:c r="Q5" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="R5" s="18" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="S5" s="17" t="str">
-        <x:v>Classic Tier 1 Slime</x:v>
+        <x:v>Passive contact-damage Tier 1 Slime</x:v>
       </x:c>
       <x:c r="T5" s="29" t="n">
         <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="U5" s="77" t="str"/>
+      <x:c r="V5" s="77" t="str">
+        <x:v>CONTACT</x:v>
+      </x:c>
+      <x:c r="W5" s="79" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X5" s="77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y5" s="77" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="Z5" s="77" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="AA5" s="77" t="n">
+        <x:v>1.8</x:v>
+      </x:c>
+      <x:c r="AB5" s="77" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>SLIME_TIER_1_ACTIVE</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>mob/0210100.img</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>7fff84d9ffda46c0a0b4f5f223a26e18</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>RootDesk/MyDesk/Models/Monsters/SlimeTier1.model</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>50faf654ee5d479cb2958edce9feaef0</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>dc932872543f4a02bf41e977ab79e5ad</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>61c27025a8f14c478f30ede1b49758bc</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>31ecb6c7cbc24599881f00cb01599f09</x:v>
+      </x:c>
+      <x:c r="J6" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="K6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L6" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="M6" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="N6" t="n">
+        <x:v>9999</x:v>
+      </x:c>
+      <x:c r="O6" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="P6" t="str">
+        <x:v>DROP_SLIME_TIER1</x:v>
+      </x:c>
+      <x:c r="Q6" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="R6" s="1" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S6" t="str">
+        <x:v>Aggressive upper-lane Slime with contact and active attack</x:v>
+      </x:c>
+      <x:c r="T6" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="U6" t="str">
+        <x:v>8b89d86b1a9c4c4288650614c6f30e67</x:v>
+      </x:c>
+      <x:c r="V6" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="W6" s="1" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y6" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="Z6" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="AA6" t="n">
+        <x:v>1.8</x:v>
+      </x:c>
+      <x:c r="AB6" t="n">
+        <x:v>0.5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1615,6 +1912,7 @@
     <x:col min="9" max="9" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="32.5" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="23.75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.5" customHeight="1">
@@ -1651,6 +1949,9 @@
       <x:c r="K1" s="20" t="str">
         <x:v>LaneKey</x:v>
       </x:c>
+      <x:c r="L1" s="68" t="str">
+        <x:v>HuntingGroundTierIndex</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -1684,6 +1985,9 @@
         <x:v>design</x:v>
       </x:c>
       <x:c r="K2" s="22" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="L2" s="70" t="str">
         <x:v>server</x:v>
       </x:c>
     </x:row>
@@ -1721,6 +2025,9 @@
       <x:c r="K3" s="25" t="str">
         <x:v>해당 스폰 그룹이 속한 전투 층 키입니다.</x:v>
       </x:c>
+      <x:c r="L3" s="73" t="str">
+        <x:v>해당 스폰 그룹이 속한 사냥터 티어 인덱스입니다.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -1756,13 +2063,16 @@
       <x:c r="K4" s="27" t="str">
         <x:v>string</x:v>
       </x:c>
+      <x:c r="L4" s="75" t="str">
+        <x:v>int</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
       <x:c r="A5" s="17" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B5" s="17" t="str">
-        <x:v>SPAWN_SLIME_TIER_1</x:v>
+        <x:v>SPAWN_SLIME_TIER_1_CENTER</x:v>
       </x:c>
       <x:c r="C5" s="17" t="n">
         <x:v>1</x:v>
@@ -1786,10 +2096,89 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J5" s="17" t="str">
-        <x:v>Single Slime foundation group</x:v>
+        <x:v>Center-lane Slime group</x:v>
       </x:c>
       <x:c r="K5" s="29" t="str">
         <x:v>CENTER</x:v>
+      </x:c>
+      <x:c r="L5" s="77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>SPAWN_SLIME_TIER_1_UPPER</x:v>
+      </x:c>
+      <x:c r="C6" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>CombatHarness/Lanes/UPPER/Spawn</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>CombatHarness/Lanes/UPPER/BoundsLeft</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>CombatHarness/Lanes/UPPER/BoundsRight</x:v>
+      </x:c>
+      <x:c r="H6" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="I6" s="1" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>Upper-lane active-attack Slime test group</x:v>
+      </x:c>
+      <x:c r="K6" t="str">
+        <x:v>UPPER</x:v>
+      </x:c>
+      <x:c r="L6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>SPAWN_SLIME_TIER_1_LOWER</x:v>
+      </x:c>
+      <x:c r="C7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>CombatHarness/Lanes/LOWER/Spawn</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>CombatHarness/Lanes/LOWER/BoundsLeft</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>CombatHarness/Lanes/LOWER/BoundsRight</x:v>
+      </x:c>
+      <x:c r="H7" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="I7" s="1" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
+        <x:v>Lower-lane Slime group</x:v>
+      </x:c>
+      <x:c r="K7" t="str">
+        <x:v>LOWER</x:v>
+      </x:c>
+      <x:c r="L7" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2016,10 +2405,10 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="H5" s="31" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I5" s="31" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J5" s="29" t="str">
         <x:v>CombatHarness/Lanes/UPPER/Spawn</x:v>
@@ -2034,7 +2423,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="N5" s="29" t="str">
-        <x:v>Future upper-lane area skill target</x:v>
+        <x:v>Upper auto-battle lane</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="16.5" customHeight="1">
@@ -2078,7 +2467,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="N6" s="29" t="str">
-        <x:v>Initial basic attack hunting lane</x:v>
+        <x:v>Initial player lane</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="16.5" customHeight="1">
@@ -2104,10 +2493,10 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="H7" s="31" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I7" s="31" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J7" s="29" t="str">
         <x:v>CombatHarness/Lanes/LOWER/Spawn</x:v>
@@ -2122,7 +2511,182 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="N7" s="29" t="str">
-        <x:v>Future lower-lane area skill target</x:v>
+        <x:v>Lower auto-battle lane</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="32.5" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="16.5" customHeight="1">
+      <x:c r="A1" s="68" t="str">
+        <x:v>CombatLaddersIndex</x:v>
+      </x:c>
+      <x:c r="B1" s="68" t="str">
+        <x:v>HuntingGroundTierIndex</x:v>
+      </x:c>
+      <x:c r="C1" s="68" t="str">
+        <x:v>MapKey</x:v>
+      </x:c>
+      <x:c r="D1" s="68" t="str">
+        <x:v>LadderKey</x:v>
+      </x:c>
+      <x:c r="E1" s="68" t="str">
+        <x:v>LowerLaneKey</x:v>
+      </x:c>
+      <x:c r="F1" s="68" t="str">
+        <x:v>UpperLaneKey</x:v>
+      </x:c>
+      <x:c r="G1" s="68" t="str">
+        <x:v>Enabled</x:v>
+      </x:c>
+      <x:c r="H1" s="68" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="16.5" customHeight="1">
+      <x:c r="A2" s="70" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="B2" s="70" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="C2" s="70" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="D2" s="70" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="E2" s="70" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="F2" s="70" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="G2" s="70" t="str">
+        <x:v>all</x:v>
+      </x:c>
+      <x:c r="H2" s="70" t="str">
+        <x:v>design</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1">
+      <x:c r="A3" s="73" t="str">
+        <x:v>층간 사다리 행을 식별하는 인덱스입니다.</x:v>
+      </x:c>
+      <x:c r="B3" s="73" t="str">
+        <x:v>HuntingGroundTiers를 참조하는 인덱스입니다.</x:v>
+      </x:c>
+      <x:c r="C3" s="73" t="str">
+        <x:v>사다리가 배치된 맵 키입니다.</x:v>
+      </x:c>
+      <x:c r="D3" s="73" t="str">
+        <x:v>맵 루트 기준 ClimbableComponent 엔티티 경로입니다.</x:v>
+      </x:c>
+      <x:c r="E3" s="73" t="str">
+        <x:v>사다리가 연결하는 아래쪽 층 키입니다.</x:v>
+      </x:c>
+      <x:c r="F3" s="73" t="str">
+        <x:v>사다리가 연결하는 위쪽 층 키입니다.</x:v>
+      </x:c>
+      <x:c r="G3" s="73" t="str">
+        <x:v>해당 사다리 경로를 사용할지 여부입니다.</x:v>
+      </x:c>
+      <x:c r="H3" s="73" t="str">
+        <x:v>기획 참고 메모입니다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="16.5" customHeight="1">
+      <x:c r="A4" s="75" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="B4" s="75" t="str">
+        <x:v>int</x:v>
+      </x:c>
+      <x:c r="C4" s="75" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D4" s="75" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="E4" s="75" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="F4" s="75" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="G4" s="75" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+      <x:c r="H4" s="75" t="str">
+        <x:v>string</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="16.5" customHeight="1">
+      <x:c r="A5" s="77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C5" s="77" t="str">
+        <x:v>map01</x:v>
+      </x:c>
+      <x:c r="D5" s="77" t="str">
+        <x:v>ladder-3</x:v>
+      </x:c>
+      <x:c r="E5" s="77" t="str">
+        <x:v>LOWER</x:v>
+      </x:c>
+      <x:c r="F5" s="77" t="str">
+        <x:v>CENTER</x:v>
+      </x:c>
+      <x:c r="G5" s="79" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H5" s="77" t="str">
+        <x:v>Lower to center ladder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="16.5" customHeight="1">
+      <x:c r="A6" s="77" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" s="77" t="str">
+        <x:v>map01</x:v>
+      </x:c>
+      <x:c r="D6" s="77" t="str">
+        <x:v>ladder-3_1</x:v>
+      </x:c>
+      <x:c r="E6" s="77" t="str">
+        <x:v>CENTER</x:v>
+      </x:c>
+      <x:c r="F6" s="77" t="str">
+        <x:v>UPPER</x:v>
+      </x:c>
+      <x:c r="G6" s="79" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H6" s="77" t="str">
+        <x:v>Center to upper ladder</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Synchronize combat actions with animation timing
</commit_message>
<xml_diff>
--- a/ExcelTable/Combat.xlsx
+++ b/ExcelTable/Combat.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatConfig" sheetId="1" r:id="Rfcc5ab25b8b24da9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuntingGroundTiers" sheetId="2" r:id="Ra9be36f89ce84f81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="3" r:id="Rff49519869bd44a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterDefinitions" sheetId="4" r:id="R74c31bae12234484"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpawnGroups" sheetId="5" r:id="R10515a0c3b954055"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLanes" sheetId="6" r:id="R35da22f3aeaa43df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLadders" sheetId="7" r:id="R54941e00c2e14a8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatConfig" sheetId="1" r:id="R5589ab23e09047c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuntingGroundTiers" sheetId="2" r:id="R9898c458704d4132"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="3" r:id="R8141985fa1ca4a53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterDefinitions" sheetId="4" r:id="R5984fac98ae6402a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpawnGroups" sheetId="5" r:id="R6913d33470dc4fa7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLanes" sheetId="6" r:id="Rcef0714457fb4455"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CombatLadders" sheetId="7" r:id="R9a546c7b9ea84e65"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -57,12 +57,37 @@
       <x:name val="Malgun Gothic"/>
     </x:font>
   </x:fonts>
-  <x:fills count="32">
+  <x:fills count="37">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF172033"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF334155"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2E8F0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -235,7 +260,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="80">
+  <x:cellXfs count="91">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
@@ -394,6 +419,19 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="32" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="32" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="33" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="33" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="34" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="34" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="34" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="35" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="35" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="36" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="36" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1087,6 +1125,9 @@
     <x:col min="14" max="14" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="23.75" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="26.25" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="26.25" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="26.25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.5" customHeight="1">
@@ -1138,6 +1179,15 @@
       <x:c r="P1" s="68" t="str">
         <x:v>LadderExitTolerance</x:v>
       </x:c>
+      <x:c r="Q1" s="81" t="str">
+        <x:v>AttackAnimationDurationSeconds</x:v>
+      </x:c>
+      <x:c r="R1" s="81" t="str">
+        <x:v>AttackHitDelaySeconds</x:v>
+      </x:c>
+      <x:c r="S1" s="81" t="str">
+        <x:v>HitAnimationDurationSeconds</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -1186,6 +1236,15 @@
         <x:v>server</x:v>
       </x:c>
       <x:c r="P2" s="70" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="Q2" s="83" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="R2" s="83" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="S2" s="83" t="str">
         <x:v>server</x:v>
       </x:c>
     </x:row>
@@ -1238,6 +1297,15 @@
       <x:c r="P3" s="73" t="str">
         <x:v>목표 층에 도착했다고 보는 세로 허용 거리입니다.</x:v>
       </x:c>
+      <x:c r="Q3" s="86" t="str">
+        <x:v>공격 행동을 잠그고 공격 애니메이션을 유지하는 전체 시간입니다.</x:v>
+      </x:c>
+      <x:c r="R3" s="86" t="str">
+        <x:v>공격 시작 후 실제 대미지를 판정하는 타격 프레임 시간입니다.</x:v>
+      </x:c>
+      <x:c r="S3" s="86" t="str">
+        <x:v>피격 행동을 잠그고 피격 애니메이션을 유지하는 시간입니다.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -1288,6 +1356,15 @@
       <x:c r="P4" s="75" t="str">
         <x:v>float</x:v>
       </x:c>
+      <x:c r="Q4" s="88" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="R4" s="88" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="S4" s="88" t="str">
+        <x:v>float</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
       <x:c r="A5" s="17" t="n">
@@ -1337,6 +1414,15 @@
       </x:c>
       <x:c r="P5" s="77" t="n">
         <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="Q5" s="90" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="R5" s="90" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
+      <x:c r="S5" s="90" t="n">
+        <x:v>0.5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1376,6 +1462,9 @@
     <x:col min="26" max="26" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="27" max="27" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="28" max="28" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="26.25" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="26.25" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="26.25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.5" customHeight="1">
@@ -1463,6 +1552,15 @@
       <x:c r="AB1" s="68" t="str">
         <x:v>ContactMoveThroughSeconds</x:v>
       </x:c>
+      <x:c r="AC1" s="81" t="str">
+        <x:v>AttackAnimationDurationSeconds</x:v>
+      </x:c>
+      <x:c r="AD1" s="81" t="str">
+        <x:v>AttackHitDelaySeconds</x:v>
+      </x:c>
+      <x:c r="AE1" s="81" t="str">
+        <x:v>HitAnimationDurationSeconds</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -1547,6 +1645,15 @@
         <x:v>server</x:v>
       </x:c>
       <x:c r="AB2" s="70" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="AC2" s="83" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="AD2" s="83" t="str">
+        <x:v>server</x:v>
+      </x:c>
+      <x:c r="AE2" s="83" t="str">
         <x:v>server</x:v>
       </x:c>
     </x:row>
@@ -1635,6 +1742,15 @@
       <x:c r="AB3" s="73" t="str">
         <x:v>접촉 피해 후 기존 방향으로 계속 이동하는 시간입니다.</x:v>
       </x:c>
+      <x:c r="AC3" s="86" t="str">
+        <x:v>공격 행동을 잠그고 공격 애니메이션을 유지하는 전체 시간입니다.</x:v>
+      </x:c>
+      <x:c r="AD3" s="86" t="str">
+        <x:v>공격 시작 후 실제 대미지를 판정하는 타격 프레임 시간입니다.</x:v>
+      </x:c>
+      <x:c r="AE3" s="86" t="str">
+        <x:v>피격 행동을 잠그고 피격 애니메이션을 유지하는 시간입니다.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -1721,6 +1837,15 @@
       <x:c r="AB4" s="75" t="str">
         <x:v>float</x:v>
       </x:c>
+      <x:c r="AC4" s="88" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="AD4" s="88" t="str">
+        <x:v>float</x:v>
+      </x:c>
+      <x:c r="AE4" s="88" t="str">
+        <x:v>float</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
       <x:c r="A5" s="17" t="n">
@@ -1805,8 +1930,17 @@
       <x:c r="AB5" s="77" t="n">
         <x:v>0.5</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6">
+      <x:c r="AC5" s="90" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="AD5" s="90" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
+      <x:c r="AE5" s="90" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="16.5" customHeight="1">
       <x:c r="A6" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -1890,6 +2024,15 @@
       </x:c>
       <x:c r="AB6" t="n">
         <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="AC6" s="90" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="AD6" s="90" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
+      <x:c r="AE6" s="90" t="n">
+        <x:v>0.35</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>